<commit_message>
No banco Tabajara finalizamos a parte 1
</commit_message>
<xml_diff>
--- a/clientes_banco_Tabajara.xlsx
+++ b/clientes_banco_Tabajara.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>extrato_bancario</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>extrato</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -471,6 +476,7 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,6 +501,7 @@
       <c r="F3" t="n">
         <v>0</v>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -517,6 +524,107 @@
         <v>402</v>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Israel albu</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>444</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>corrente</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>403</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>jose</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4444</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>salario</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>404</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jof</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>444</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>corrente</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>405</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jesura</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>555</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>corrente</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>406</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nesta aula fizemos a parte dois do banco tabajara, porem termos que fazer um FOR para percorrer as linha do excel
</commit_message>
<xml_diff>
--- a/clientes_banco_Tabajara.xlsx
+++ b/clientes_banco_Tabajara.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,11 +444,6 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>extrato_bancario</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>extrato</t>
         </is>
       </c>
@@ -476,20 +471,19 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Israel V</t>
+          <t>Heloisa</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5555</v>
+        <v>55555</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>corrente</t>
+          <t>Salario</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -499,132 +493,6 @@
         <v>401</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Helo</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2222</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Salario</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="n">
-        <v>402</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Israel albu</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>444</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>corrente</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>403</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>jose</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>4444</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>salario</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="n">
-        <v>404</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Jof</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>444</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>corrente</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>405</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Jesura</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>555</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>corrente</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" t="n">
-        <v>406</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>